<commit_message>
update format and fix tracking
</commit_message>
<xml_diff>
--- a/templates/PhieuKetQua.xlsx
+++ b/templates/PhieuKetQua.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/congdat/Developer/lab-admin-go/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E604262C-7D94-0642-A9FD-B123E2502B64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63EE3EA5-3DF8-254D-8C6D-19D87FBAAB9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10760" yWindow="6440" windowWidth="27640" windowHeight="15160" xr2:uid="{8AF87BAE-0B61-4E46-A5C8-CBD3A6B78A3F}"/>
+    <workbookView xWindow="2600" yWindow="4480" windowWidth="27640" windowHeight="15160" xr2:uid="{8AF87BAE-0B61-4E46-A5C8-CBD3A6B78A3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Ngày:</t>
   </si>
@@ -92,6 +92,9 @@
   </si>
   <si>
     <t xml:space="preserve">PHÒNG XÉT NGHIỆM </t>
+  </si>
+  <si>
+    <t>CKI.XN NGUYỄN CÔNG MẪN</t>
   </si>
 </sst>
 </file>
@@ -101,7 +104,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -138,6 +141,13 @@
     <font>
       <b/>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <name val="Myriad pro"/>
     </font>
   </fonts>
@@ -176,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -225,6 +235,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -572,7 +585,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:F10"/>
+  <dimension ref="B1:F15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="1.83203125" customWidth="1"/>
@@ -645,7 +658,7 @@
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="2:6" ht="30">
+    <row r="7" spans="2:6" ht="32">
       <c r="B7" s="6" t="s">
         <v>11</v>
       </c>
@@ -676,17 +689,25 @@
       <c r="E9" s="12"/>
       <c r="F9" s="11"/>
     </row>
-    <row r="10" spans="2:6">
+    <row r="10" spans="2:6" ht="18">
       <c r="B10" s="14"/>
       <c r="C10" s="14"/>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+    </row>
+    <row r="15" spans="2:6">
+      <c r="D15" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="D15:F15"/>
     <mergeCell ref="D10:F10"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="E3:F3"/>

</xml_diff>

<commit_message>
feat: support export report file in PDF format (#26)
* update format and fix tracking

* update format and print area

* support export report in PDF format

* add makefile rule
</commit_message>
<xml_diff>
--- a/templates/PhieuKetQua.xlsx
+++ b/templates/PhieuKetQua.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/congdat/Developer/lab-admin-go/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E604262C-7D94-0642-A9FD-B123E2502B64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63EE3EA5-3DF8-254D-8C6D-19D87FBAAB9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10760" yWindow="6440" windowWidth="27640" windowHeight="15160" xr2:uid="{8AF87BAE-0B61-4E46-A5C8-CBD3A6B78A3F}"/>
+    <workbookView xWindow="2600" yWindow="4480" windowWidth="27640" windowHeight="15160" xr2:uid="{8AF87BAE-0B61-4E46-A5C8-CBD3A6B78A3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Ngày:</t>
   </si>
@@ -92,6 +92,9 @@
   </si>
   <si>
     <t xml:space="preserve">PHÒNG XÉT NGHIỆM </t>
+  </si>
+  <si>
+    <t>CKI.XN NGUYỄN CÔNG MẪN</t>
   </si>
 </sst>
 </file>
@@ -101,7 +104,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -138,6 +141,13 @@
     <font>
       <b/>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <name val="Myriad pro"/>
     </font>
   </fonts>
@@ -176,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -225,6 +235,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -572,7 +585,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:F10"/>
+  <dimension ref="B1:F15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="1.83203125" customWidth="1"/>
@@ -645,7 +658,7 @@
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="2:6" ht="30">
+    <row r="7" spans="2:6" ht="32">
       <c r="B7" s="6" t="s">
         <v>11</v>
       </c>
@@ -676,17 +689,25 @@
       <c r="E9" s="12"/>
       <c r="F9" s="11"/>
     </row>
-    <row r="10" spans="2:6">
+    <row r="10" spans="2:6" ht="18">
       <c r="B10" s="14"/>
       <c r="C10" s="14"/>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+    </row>
+    <row r="15" spans="2:6">
+      <c r="D15" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="D15:F15"/>
     <mergeCell ref="D10:F10"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="E3:F3"/>

</xml_diff>

<commit_message>
feat: update report format (#44)
</commit_message>
<xml_diff>
--- a/templates/PhieuKetQua.xlsx
+++ b/templates/PhieuKetQua.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/congdat/Developer/lab-admin-go/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63EE3EA5-3DF8-254D-8C6D-19D87FBAAB9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F037EC33-4271-B74D-A91E-7BD431019E8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2600" yWindow="4480" windowWidth="27640" windowHeight="15160" xr2:uid="{8AF87BAE-0B61-4E46-A5C8-CBD3A6B78A3F}"/>
   </bookViews>
@@ -140,14 +140,13 @@
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
+      <sz val="14"/>
+      <name val="Myriad pro"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
+      <color theme="1"/>
       <name val="Myriad pro"/>
     </font>
   </fonts>
@@ -589,10 +588,10 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="1.83203125" customWidth="1"/>
-    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="2" max="2" width="9.83203125" customWidth="1"/>
     <col min="3" max="3" width="37.6640625" customWidth="1"/>
     <col min="4" max="4" width="16.5" customWidth="1"/>
-    <col min="5" max="5" width="10.1640625" customWidth="1"/>
+    <col min="5" max="5" width="13.83203125" customWidth="1"/>
     <col min="6" max="6" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -692,18 +691,18 @@
     <row r="10" spans="2:6" ht="18">
       <c r="B10" s="14"/>
       <c r="C10" s="14"/>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-    </row>
-    <row r="15" spans="2:6">
-      <c r="D15" s="15" t="s">
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+    </row>
+    <row r="15" spans="2:6" ht="18">
+      <c r="D15" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>